<commit_message>
full code before deleting
</commit_message>
<xml_diff>
--- a/Data/yield_reduction_contribution.xlsx
+++ b/Data/yield_reduction_contribution.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ximinpiao/Documents/GitHub/UTR-Soybean-BioCro/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F26E82-E6B6-924B-9070-FAAE3844AC80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDC5A7CB-401D-3B42-8DB9-285004D0C9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-7340" windowWidth="51200" windowHeight="28200" activeTab="1" xr2:uid="{A8BE2E2B-28B6-A944-AF5D-F88762CA8258}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{A8BE2E2B-28B6-A944-AF5D-F88762CA8258}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Proulx" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
+    <sheet name="Carrera" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="66">
   <si>
     <t>Treatment</t>
   </si>
@@ -132,10 +133,6 @@
   </si>
   <si>
     <t>% Reduction
-Grain Yield</t>
-  </si>
-  <si>
-    <t>% Reduction
 Grain Number</t>
   </si>
   <si>
@@ -159,17 +156,107 @@
   </si>
   <si>
     <t>(Validation)</t>
+  </si>
+  <si>
+    <t>Defoliation timing</t>
+  </si>
+  <si>
+    <t>Exp 1 – MG2</t>
+  </si>
+  <si>
+    <t>Exp 2 – MG4</t>
+  </si>
+  <si>
+    <t>Seed wt% change</t>
+  </si>
+  <si>
+    <t>Pod wt% change</t>
+  </si>
+  <si>
+    <t>V4</t>
+  </si>
+  <si>
+    <t>−19%</t>
+  </si>
+  <si>
+    <t>−13%</t>
+  </si>
+  <si>
+    <t>ns</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>−17%</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>−14%</t>
+  </si>
+  <si>
+    <t>−12%</t>
+  </si>
+  <si>
+    <t>R5+1wk</t>
+  </si>
+  <si>
+    <t>−29%</t>
+  </si>
+  <si>
+    <t>−21%</t>
+  </si>
+  <si>
+    <t>−22%</t>
+  </si>
+  <si>
+    <t>R5+2wk</t>
+  </si>
+  <si>
+    <t>−32%</t>
+  </si>
+  <si>
+    <t>R5+3wk</t>
+  </si>
+  <si>
+    <t>R5+4wk</t>
+  </si>
+  <si>
+    <t>seed:pod ratio change</t>
+  </si>
+  <si>
+    <t>% Reduction Seed:Pod ratio*</t>
+  </si>
+  <si>
+    <t>% Reduction
+Yield</t>
+  </si>
+  <si>
+    <t>* % Reduction in Seed:Pod ratio=1-(1-%Reduction Yield)/((1-%Reduction Grain Number)*(1-0.76*%Reduction in Grain Weight)</t>
+  </si>
+  <si>
+    <t>Pod = Number of Pods * Unit Pod weight</t>
+  </si>
+  <si>
+    <t>% Reduction in Number of Pods = % Reduction Grain Number</t>
+  </si>
+  <si>
+    <t>% Reduction in Unit Pod weight = 1 - 76% * Reduction in Unit Grain weight</t>
+  </si>
+  <si>
+    <t>76% seed:pod ratio is found in the SoyFACE data.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="0.0\%"/>
-    <numFmt numFmtId="171" formatCode="0.0%"/>
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -221,6 +308,14 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -312,18 +407,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -339,19 +428,26 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="7" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -954,7 +1050,7 @@
         <v>-8.2872928176795577E-2</v>
       </c>
       <c r="G11" s="2">
-        <f t="shared" si="0"/>
+        <f>C11 *E11 / 100 * 10^4 / 10^6</f>
         <v>3.0544000000000007</v>
       </c>
       <c r="H11" s="2">
@@ -1197,8 +1293,207 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF0CB73A-0032-5140-B1AB-CEB4A49D699E}">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B2" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="17"/>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="17">
+        <f>0.14</f>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="17">
+        <f>1-84/88</f>
+        <v>4.5454545454545414E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="17">
+        <f>1-0.71/0.79</f>
+        <v>0.10126582278481022</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="17">
+        <f>1-78/88</f>
+        <v>0.11363636363636365</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D53ECF1-E7CD-2548-95A4-57BCCF098550}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1206,582 +1501,661 @@
     <col min="5" max="6" width="16" customWidth="1"/>
     <col min="7" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="25.6640625" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-    </row>
-    <row r="3" spans="1:11" ht="28" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+    </row>
+    <row r="3" spans="1:11" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="J3" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="7">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7">
+        <v>542</v>
+      </c>
+      <c r="E4" s="7">
+        <v>2737</v>
+      </c>
+      <c r="F4" s="7">
+        <v>198.6</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="H4" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="7" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="9">
+      <c r="K4" s="7"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="8">
         <v>1</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="9">
-        <v>0</v>
-      </c>
-      <c r="D4" s="9">
-        <v>542</v>
-      </c>
-      <c r="E4" s="9">
-        <v>2737</v>
-      </c>
-      <c r="F4" s="9">
-        <v>198.6</v>
-      </c>
-      <c r="G4" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="10">
-        <v>1</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <v>33</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="8">
         <v>511</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="8">
         <v>2612</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="8">
         <v>195.9</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="11">
         <f>($D$4-D5)/$D$4</f>
         <v>5.719557195571956E-2</v>
       </c>
-      <c r="H5" s="14">
+      <c r="H5" s="10">
         <f>($E$4-E5)/$E$4</f>
         <v>4.5670442089879429E-2</v>
       </c>
-      <c r="I5" s="15">
+      <c r="I5" s="11">
         <f>($F$5-F5)/$F$5</f>
         <v>0</v>
       </c>
-      <c r="J5" s="15">
+      <c r="J5" s="11">
         <f>1-(1-H5)*(1-I5)</f>
         <v>4.5670442089879471E-2</v>
       </c>
-      <c r="K5" s="13"/>
+      <c r="K5" s="11">
+        <f>1-(1-G5)/((1-H5)*(1-0.76*I5))</f>
+        <v>1.2076677045484097E-2</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="10">
+      <c r="A6" s="8">
         <v>1</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="10">
+      <c r="B6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="8">
         <v>66</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>444</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="8">
         <v>2361</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="8">
         <v>189.1</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="11">
         <f t="shared" ref="G6:G10" si="0">($D$4-D6)/$D$4</f>
         <v>0.18081180811808117</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="10">
         <f t="shared" ref="H6:H10" si="1">($E$4-E6)/$E$4</f>
         <v>0.13737668980635734</v>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="11">
         <f t="shared" ref="I6:I10" si="2">($F$5-F6)/$F$5</f>
         <v>3.4711587544665704E-2</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="11">
         <f t="shared" ref="J6:J17" si="3">1-(1-H6)*(1-I6)</f>
         <v>0.16731971435621329</v>
       </c>
+      <c r="K6" s="11">
+        <f t="shared" ref="K6:K10" si="4">1-(1-G6)/((1-H6)*(1-0.76*I6))</f>
+        <v>2.4621075977793061E-2</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="10">
+      <c r="A7" s="8">
         <v>1</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="10">
+      <c r="B7" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="8">
         <v>100</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="8">
         <v>170</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="8">
         <v>1658</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="8">
         <v>102.9</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="11">
         <f t="shared" si="0"/>
         <v>0.68634686346863472</v>
       </c>
-      <c r="H7" s="14">
+      <c r="H7" s="10">
         <f t="shared" si="1"/>
         <v>0.39422725611983922</v>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="11">
         <f t="shared" si="2"/>
         <v>0.47473200612557426</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="11">
         <f t="shared" si="3"/>
         <v>0.68180696607826152</v>
       </c>
+      <c r="K7" s="11">
+        <f>1-(1-G7)/((1-H7)*(1-0.76*I7))</f>
+        <v>0.18997085980276485</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="10">
+      <c r="A8" s="8">
         <v>1</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="8">
         <v>33</v>
       </c>
-      <c r="C8" s="10">
-        <v>33</v>
-      </c>
-      <c r="D8" s="10">
+      <c r="D8" s="8">
         <v>537</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="8">
         <v>2877</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="8">
         <v>186.7</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="11">
         <f t="shared" si="0"/>
         <v>9.2250922509225092E-3</v>
       </c>
-      <c r="H8" s="14">
+      <c r="H8" s="10">
         <f>($E$4-E8)/$E$4</f>
         <v>-5.1150895140664961E-2</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="11">
         <f t="shared" si="2"/>
         <v>4.696273608984184E-2</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="11">
         <f t="shared" si="3"/>
         <v>-1.7859730615730207E-3</v>
       </c>
+      <c r="K8" s="11">
+        <f t="shared" si="4"/>
+        <v>2.2551193686457749E-2</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="10">
+      <c r="A9" s="8">
         <v>1</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="10">
+      <c r="B9" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="8">
         <v>66</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="8">
         <v>437</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="8">
         <v>2574</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="8">
         <v>171.6</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="11">
         <f t="shared" si="0"/>
         <v>0.19372693726937271</v>
       </c>
-      <c r="H9" s="14">
+      <c r="H9" s="10">
         <f t="shared" si="1"/>
         <v>5.9554256485202774E-2</v>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="11">
         <f t="shared" si="2"/>
         <v>0.12404287901990817</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="11">
         <f t="shared" si="3"/>
         <v>0.17620985407279632</v>
       </c>
+      <c r="K9" s="11">
+        <f t="shared" si="4"/>
+        <v>5.3434016332437273E-2</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="10">
+      <c r="A10" s="8">
         <v>1</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="10">
+      <c r="B10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="8">
         <v>100</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="8">
         <v>249</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="8">
         <v>2347</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="8">
         <v>106.6</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="11">
         <f t="shared" si="0"/>
         <v>0.54059040590405905</v>
       </c>
-      <c r="H10" s="14">
+      <c r="H10" s="10">
         <f t="shared" si="1"/>
         <v>0.14249177932042381</v>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="11">
         <f t="shared" si="2"/>
         <v>0.45584481878509447</v>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="11">
         <f t="shared" si="3"/>
         <v>0.53338245878283408</v>
       </c>
+      <c r="K10" s="11">
+        <f t="shared" si="4"/>
+        <v>0.18025707953719772</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="9">
+      <c r="A11" s="7">
         <v>2</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="7">
         <v>0</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="7">
         <v>446</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="7">
         <v>2672</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="7">
         <v>167.1</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="K11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="9">
+        <v>2</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="11">
-        <v>2</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="11">
+      <c r="C12" s="9">
         <v>33</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="9">
         <v>385</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="9">
         <v>2535</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="9">
         <v>151.69999999999999</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="11">
         <f>($D$11-D12)/$D$11</f>
         <v>0.1367713004484305</v>
       </c>
-      <c r="H12" s="14">
+      <c r="H12" s="10">
         <f>($E$11-E12)/$E$11</f>
         <v>5.1272455089820361E-2</v>
       </c>
-      <c r="I12" s="15">
+      <c r="I12" s="11">
         <f>($F$11-F12)/$F$11</f>
         <v>9.2160383004189148E-2</v>
       </c>
-      <c r="J12" s="15">
+      <c r="J12" s="11">
         <f>1-(1-H12)*(1-I12)</f>
         <v>0.13870754899536664</v>
       </c>
+      <c r="K12" s="11">
+        <f>1-(1-G12)/((1-H12)*(1-0.76*I12))</f>
+        <v>2.158979177808984E-2</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="11">
+      <c r="A13" s="9">
         <v>2</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="11">
+      <c r="B13" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="9">
         <v>66</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="9">
         <v>340</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="9">
         <v>2154</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="9">
         <v>159.6</v>
       </c>
-      <c r="G13" s="15">
-        <f t="shared" ref="G13:G17" si="4">($D$11-D13)/$D$11</f>
+      <c r="G13" s="11">
+        <f t="shared" ref="G13:G17" si="5">($D$11-D13)/$D$11</f>
         <v>0.23766816143497757</v>
       </c>
-      <c r="H13" s="14">
-        <f t="shared" ref="H13:H17" si="5">($E$11-E13)/$E$11</f>
+      <c r="H13" s="10">
+        <f t="shared" ref="H13:H17" si="6">($E$11-E13)/$E$11</f>
         <v>0.19386227544910178</v>
       </c>
-      <c r="I13" s="15">
-        <f t="shared" ref="I13:I17" si="6">($F$11-F13)/$F$11</f>
+      <c r="I13" s="11">
+        <f t="shared" ref="I13:I17" si="7">($F$11-F13)/$F$11</f>
         <v>4.4883303411131059E-2</v>
       </c>
-      <c r="J13" s="15">
+      <c r="J13" s="11">
         <f t="shared" si="3"/>
         <v>0.23004439953127853</v>
       </c>
+      <c r="K13" s="11">
+        <f>1-(1-G13)/((1-H13)*(1-0.76*I13))</f>
+        <v>2.0943550458836002E-2</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="11">
+      <c r="A14" s="9">
         <v>2</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="11">
+      <c r="B14" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="9">
         <v>100</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="9">
         <v>108</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="9">
         <v>1342</v>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="9">
         <v>81.5</v>
       </c>
-      <c r="G14" s="15">
-        <f t="shared" si="4"/>
+      <c r="G14" s="11">
+        <f t="shared" si="5"/>
         <v>0.75784753363228696</v>
       </c>
-      <c r="H14" s="14">
-        <f t="shared" si="5"/>
+      <c r="H14" s="10">
+        <f t="shared" si="6"/>
         <v>0.4977544910179641</v>
       </c>
-      <c r="I14" s="15">
-        <f t="shared" si="6"/>
+      <c r="I14" s="11">
+        <f t="shared" si="7"/>
         <v>0.51226810293237579</v>
       </c>
-      <c r="J14" s="15">
+      <c r="J14" s="11">
         <f t="shared" si="3"/>
         <v>0.75503884511049713</v>
       </c>
+      <c r="K14" s="11">
+        <f t="shared" ref="K13:K17" si="8">1-(1-G14)/((1-H14)*(1-0.76*I14))</f>
+        <v>0.2104824095088067</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="11">
+      <c r="A15" s="9">
         <v>2</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="9">
         <v>33</v>
       </c>
-      <c r="C15" s="11">
-        <v>33</v>
-      </c>
-      <c r="D15" s="11">
+      <c r="D15" s="9">
         <v>348</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="9">
         <v>2256</v>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="9">
         <v>154.1</v>
       </c>
-      <c r="G15" s="15">
-        <f t="shared" si="4"/>
+      <c r="G15" s="11">
+        <f t="shared" si="5"/>
         <v>0.21973094170403587</v>
       </c>
-      <c r="H15" s="14">
-        <f t="shared" si="5"/>
+      <c r="H15" s="10">
+        <f t="shared" si="6"/>
         <v>0.15568862275449102</v>
       </c>
-      <c r="I15" s="15">
-        <f t="shared" si="6"/>
+      <c r="I15" s="11">
+        <f t="shared" si="7"/>
         <v>7.7797725912627166E-2</v>
       </c>
-      <c r="J15" s="15">
+      <c r="J15" s="11">
         <f t="shared" si="3"/>
         <v>0.2213741278663498</v>
       </c>
+      <c r="K15" s="11">
+        <f t="shared" si="8"/>
+        <v>1.7776316509562573E-2</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="11">
+      <c r="A16" s="9">
         <v>2</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" s="11">
+      <c r="B16" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="9">
         <v>66</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="9">
         <v>311</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="9">
         <v>2220</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="9">
         <v>140.1</v>
       </c>
-      <c r="G16" s="15">
-        <f t="shared" si="4"/>
+      <c r="G16" s="11">
+        <f t="shared" si="5"/>
         <v>0.30269058295964124</v>
       </c>
-      <c r="H16" s="14">
-        <f t="shared" si="5"/>
+      <c r="H16" s="10">
+        <f t="shared" si="6"/>
         <v>0.16916167664670659</v>
       </c>
-      <c r="I16" s="15">
-        <f t="shared" si="6"/>
+      <c r="I16" s="11">
+        <f t="shared" si="7"/>
         <v>0.16157989228007183</v>
       </c>
-      <c r="J16" s="15">
+      <c r="J16" s="11">
         <f t="shared" si="3"/>
         <v>0.30340844343628726</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="11">
+      <c r="K16" s="11">
+        <f t="shared" si="8"/>
+        <v>4.3222965949012315E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="9">
         <v>2</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="11">
+      <c r="B17" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="9">
         <v>100</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="9">
         <v>240</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="9">
         <v>2174</v>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="9">
         <v>111.2</v>
       </c>
-      <c r="G17" s="15">
-        <f t="shared" si="4"/>
+      <c r="G17" s="11">
+        <f t="shared" si="5"/>
         <v>0.46188340807174888</v>
       </c>
-      <c r="H17" s="14">
-        <f t="shared" si="5"/>
+      <c r="H17" s="10">
+        <f t="shared" si="6"/>
         <v>0.18637724550898205</v>
       </c>
-      <c r="I17" s="15">
-        <f t="shared" si="6"/>
+      <c r="I17" s="11">
+        <f t="shared" si="7"/>
         <v>0.33453022142429678</v>
       </c>
-      <c r="J17" s="15">
+      <c r="J17" s="11">
         <f t="shared" si="3"/>
         <v>0.4585586457247085</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
+      <c r="K17" s="11">
+        <f t="shared" si="8"/>
+        <v>0.11313821793777645</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>65</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>